<commit_message>
feat(templates): complete per-month templates to all 12 months
Staff shipped only MAC-DISEMBER (no Jan/Feb) and student had gaps too. Add the
missing months by cloning a month sheet (exact styling + the bordered data
grid) and swapping the month in the title, ordered JANUARI..DISEMBER. Staff and
student templates now each have 12 month tabs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Pelajar.xlsx
+++ b/assets/templates/Pelajar.xlsx
@@ -15,10 +15,13 @@
   <sheets>
     <sheet name="JANUARI" sheetId="16" r:id="rId1"/>
     <sheet name="FEBRUARI" sheetId="17" r:id="rId2"/>
+    <sheet name="MAC" sheetId="18" r:id="rId14"/>
     <sheet name="APRIL" sheetId="6" r:id="rId3"/>
     <sheet name="MEI" sheetId="7" r:id="rId4"/>
     <sheet name="JUN" sheetId="9" r:id="rId5"/>
     <sheet name="JULAI" sheetId="10" r:id="rId6"/>
+    <sheet name="OGOS" sheetId="19" r:id="rId15"/>
+    <sheet name="SEPTEMBER" sheetId="20" r:id="rId16"/>
     <sheet name="OKTOBER" sheetId="11" r:id="rId7"/>
     <sheet name="NOVEMBER" sheetId="13" r:id="rId8"/>
     <sheet name="DISEMBER" sheetId="15" r:id="rId9"/>
@@ -1983,6 +1986,1884 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB8B4E8A-7EF6-443B-9F61-C7CAEBB32554}">
+  <dimension ref="A1:I52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="53" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" style="53" customWidth="1"/>
+    <col min="12" max="12" width="24.140625" style="47" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MAKLUMAN PELEKAT KENDERAAN PELAJAR BULAN MAC TAHUN 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+    </row>
+    <row r="2" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="67" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="48"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="112"/>
+      <c r="B3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="112"/>
+      <c r="B4" s="112"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="112"/>
+      <c r="E4" s="112"/>
+      <c r="F4" s="112"/>
+      <c r="G4" s="112"/>
+      <c r="H4" s="112"/>
+      <c r="I4" s="112"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="112"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="112"/>
+      <c r="E5" s="112"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="112"/>
+      <c r="H5" s="112"/>
+      <c r="I5" s="112"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="112"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="112"/>
+      <c r="G6" s="112"/>
+      <c r="H6" s="112"/>
+      <c r="I6" s="112"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="112"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="112"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="112"/>
+      <c r="H7" s="112"/>
+      <c r="I7" s="112"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="112"/>
+      <c r="B8" s="112"/>
+      <c r="C8" s="112"/>
+      <c r="D8" s="112"/>
+      <c r="E8" s="112"/>
+      <c r="F8" s="112"/>
+      <c r="G8" s="112"/>
+      <c r="H8" s="112"/>
+      <c r="I8" s="112"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="112"/>
+      <c r="B9" s="112"/>
+      <c r="C9" s="112"/>
+      <c r="D9" s="112"/>
+      <c r="E9" s="112"/>
+      <c r="F9" s="112"/>
+      <c r="G9" s="112"/>
+      <c r="H9" s="112"/>
+      <c r="I9" s="112"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="112"/>
+      <c r="B10" s="112"/>
+      <c r="C10" s="112"/>
+      <c r="D10" s="112"/>
+      <c r="E10" s="112"/>
+      <c r="F10" s="112"/>
+      <c r="G10" s="112"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="112"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
+      <c r="G11" s="112"/>
+      <c r="H11" s="112"/>
+      <c r="I11" s="112"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="112"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
+      <c r="G12" s="112"/>
+      <c r="H12" s="112"/>
+      <c r="I12" s="112"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="112"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="112"/>
+      <c r="H13" s="112"/>
+      <c r="I13" s="112"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="112"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
+      <c r="G14" s="112"/>
+      <c r="H14" s="112"/>
+      <c r="I14" s="112"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="112"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="112"/>
+      <c r="I15" s="112"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="112"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
+      <c r="G16" s="112"/>
+      <c r="H16" s="112"/>
+      <c r="I16" s="112"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="112"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="112"/>
+      <c r="I17" s="112"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="112"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
+      <c r="G18" s="112"/>
+      <c r="H18" s="112"/>
+      <c r="I18" s="112"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="112"/>
+      <c r="B19" s="112"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
+      <c r="G19" s="112"/>
+      <c r="H19" s="112"/>
+      <c r="I19" s="112"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="112"/>
+      <c r="B20" s="112"/>
+      <c r="C20" s="112"/>
+      <c r="D20" s="112"/>
+      <c r="E20" s="112"/>
+      <c r="F20" s="112"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="112"/>
+      <c r="I20" s="112"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="112"/>
+      <c r="B21" s="112"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="112"/>
+      <c r="E21" s="112"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="112"/>
+      <c r="H21" s="112"/>
+      <c r="I21" s="112"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="112"/>
+      <c r="B22" s="112"/>
+      <c r="C22" s="112"/>
+      <c r="D22" s="112"/>
+      <c r="E22" s="112"/>
+      <c r="F22" s="112"/>
+      <c r="G22" s="112"/>
+      <c r="H22" s="112"/>
+      <c r="I22" s="112"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="112"/>
+      <c r="B23" s="112"/>
+      <c r="C23" s="112"/>
+      <c r="D23" s="112"/>
+      <c r="E23" s="112"/>
+      <c r="F23" s="112"/>
+      <c r="G23" s="112"/>
+      <c r="H23" s="112"/>
+      <c r="I23" s="112"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="112"/>
+      <c r="B24" s="112"/>
+      <c r="C24" s="112"/>
+      <c r="D24" s="112"/>
+      <c r="E24" s="112"/>
+      <c r="F24" s="112"/>
+      <c r="G24" s="112"/>
+      <c r="H24" s="112"/>
+      <c r="I24" s="112"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="112"/>
+      <c r="B25" s="112"/>
+      <c r="C25" s="112"/>
+      <c r="D25" s="112"/>
+      <c r="E25" s="112"/>
+      <c r="F25" s="112"/>
+      <c r="G25" s="112"/>
+      <c r="H25" s="112"/>
+      <c r="I25" s="112"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="112"/>
+      <c r="B26" s="112"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
+      <c r="E26" s="112"/>
+      <c r="F26" s="112"/>
+      <c r="G26" s="112"/>
+      <c r="H26" s="112"/>
+      <c r="I26" s="112"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="112"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
+      <c r="F27" s="112"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="112"/>
+      <c r="I27" s="112"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="112"/>
+      <c r="B28" s="112"/>
+      <c r="C28" s="112"/>
+      <c r="D28" s="112"/>
+      <c r="E28" s="112"/>
+      <c r="F28" s="112"/>
+      <c r="G28" s="112"/>
+      <c r="H28" s="112"/>
+      <c r="I28" s="112"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="112"/>
+      <c r="B29" s="112"/>
+      <c r="C29" s="112"/>
+      <c r="D29" s="112"/>
+      <c r="E29" s="112"/>
+      <c r="F29" s="112"/>
+      <c r="G29" s="112"/>
+      <c r="H29" s="112"/>
+      <c r="I29" s="112"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="112"/>
+      <c r="B30" s="112"/>
+      <c r="C30" s="112"/>
+      <c r="D30" s="112"/>
+      <c r="E30" s="112"/>
+      <c r="F30" s="112"/>
+      <c r="G30" s="112"/>
+      <c r="H30" s="112"/>
+      <c r="I30" s="112"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="112"/>
+      <c r="B31" s="112"/>
+      <c r="C31" s="112"/>
+      <c r="D31" s="112"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="112"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="112"/>
+      <c r="I31" s="112"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="112"/>
+      <c r="B32" s="112"/>
+      <c r="C32" s="112"/>
+      <c r="D32" s="112"/>
+      <c r="E32" s="112"/>
+      <c r="F32" s="112"/>
+      <c r="G32" s="112"/>
+      <c r="H32" s="112"/>
+      <c r="I32" s="112"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="112"/>
+      <c r="B33" s="112"/>
+      <c r="C33" s="112"/>
+      <c r="D33" s="112"/>
+      <c r="E33" s="112"/>
+      <c r="F33" s="112"/>
+      <c r="G33" s="112"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="112"/>
+      <c r="B34" s="112"/>
+      <c r="C34" s="112"/>
+      <c r="D34" s="112"/>
+      <c r="E34" s="112"/>
+      <c r="F34" s="112"/>
+      <c r="G34" s="112"/>
+      <c r="H34" s="112"/>
+      <c r="I34" s="112"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="112"/>
+      <c r="B35" s="112"/>
+      <c r="C35" s="112"/>
+      <c r="D35" s="112"/>
+      <c r="E35" s="112"/>
+      <c r="F35" s="112"/>
+      <c r="G35" s="112"/>
+      <c r="H35" s="112"/>
+      <c r="I35" s="112"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="112"/>
+      <c r="B36" s="112"/>
+      <c r="C36" s="112"/>
+      <c r="D36" s="112"/>
+      <c r="E36" s="112"/>
+      <c r="F36" s="112"/>
+      <c r="G36" s="112"/>
+      <c r="H36" s="112"/>
+      <c r="I36" s="112"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="112"/>
+      <c r="B37" s="112"/>
+      <c r="C37" s="112"/>
+      <c r="D37" s="112"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="112"/>
+      <c r="G37" s="112"/>
+      <c r="H37" s="112"/>
+      <c r="I37" s="112"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="112"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
+      <c r="G38" s="112"/>
+      <c r="H38" s="112"/>
+      <c r="I38" s="112"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="112"/>
+      <c r="B39" s="112"/>
+      <c r="C39" s="112"/>
+      <c r="D39" s="112"/>
+      <c r="E39" s="112"/>
+      <c r="F39" s="112"/>
+      <c r="G39" s="112"/>
+      <c r="H39" s="112"/>
+      <c r="I39" s="112"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="112"/>
+      <c r="B40" s="112"/>
+      <c r="C40" s="112"/>
+      <c r="D40" s="112"/>
+      <c r="E40" s="112"/>
+      <c r="F40" s="112"/>
+      <c r="G40" s="112"/>
+      <c r="H40" s="112"/>
+      <c r="I40" s="112"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="112"/>
+      <c r="B41" s="112"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="112"/>
+      <c r="G41" s="112"/>
+      <c r="H41" s="112"/>
+      <c r="I41" s="112"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="112"/>
+      <c r="B42" s="112"/>
+      <c r="C42" s="112"/>
+      <c r="D42" s="112"/>
+      <c r="E42" s="112"/>
+      <c r="F42" s="112"/>
+      <c r="G42" s="112"/>
+      <c r="H42" s="112"/>
+      <c r="I42" s="112"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="112"/>
+      <c r="B43" s="112"/>
+      <c r="C43" s="112"/>
+      <c r="D43" s="112"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="112"/>
+      <c r="G43" s="112"/>
+      <c r="H43" s="112"/>
+      <c r="I43" s="112"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="112"/>
+      <c r="B44" s="112"/>
+      <c r="C44" s="112"/>
+      <c r="D44" s="112"/>
+      <c r="E44" s="112"/>
+      <c r="F44" s="112"/>
+      <c r="G44" s="112"/>
+      <c r="H44" s="112"/>
+      <c r="I44" s="112"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="112"/>
+      <c r="B45" s="112"/>
+      <c r="C45" s="112"/>
+      <c r="D45" s="112"/>
+      <c r="E45" s="112"/>
+      <c r="F45" s="112"/>
+      <c r="G45" s="112"/>
+      <c r="H45" s="112"/>
+      <c r="I45" s="112"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="112"/>
+      <c r="B46" s="112"/>
+      <c r="C46" s="112"/>
+      <c r="D46" s="112"/>
+      <c r="E46" s="112"/>
+      <c r="F46" s="112"/>
+      <c r="G46" s="112"/>
+      <c r="H46" s="112"/>
+      <c r="I46" s="112"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="112"/>
+      <c r="B47" s="112"/>
+      <c r="C47" s="112"/>
+      <c r="D47" s="112"/>
+      <c r="E47" s="112"/>
+      <c r="F47" s="112"/>
+      <c r="G47" s="112"/>
+      <c r="H47" s="112"/>
+      <c r="I47" s="112"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="112"/>
+      <c r="B48" s="112"/>
+      <c r="C48" s="112"/>
+      <c r="D48" s="112"/>
+      <c r="E48" s="112"/>
+      <c r="F48" s="112"/>
+      <c r="G48" s="112"/>
+      <c r="H48" s="112"/>
+      <c r="I48" s="112"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="112"/>
+      <c r="B49" s="112"/>
+      <c r="C49" s="112"/>
+      <c r="D49" s="112"/>
+      <c r="E49" s="112"/>
+      <c r="F49" s="112"/>
+      <c r="G49" s="112"/>
+      <c r="H49" s="112"/>
+      <c r="I49" s="112"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="112"/>
+      <c r="B50" s="112"/>
+      <c r="C50" s="112"/>
+      <c r="D50" s="112"/>
+      <c r="E50" s="112"/>
+      <c r="F50" s="112"/>
+      <c r="G50" s="112"/>
+      <c r="H50" s="112"/>
+      <c r="I50" s="112"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="112"/>
+      <c r="B51" s="112"/>
+      <c r="C51" s="112"/>
+      <c r="D51" s="112"/>
+      <c r="E51" s="112"/>
+      <c r="F51" s="112"/>
+      <c r="G51" s="112"/>
+      <c r="H51" s="112"/>
+      <c r="I51" s="112"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="112"/>
+      <c r="B52" s="112"/>
+      <c r="C52" s="112"/>
+      <c r="D52" s="112"/>
+      <c r="E52" s="112"/>
+      <c r="F52" s="112"/>
+      <c r="G52" s="112"/>
+      <c r="H52" s="112"/>
+      <c r="I52" s="112"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB8B4E8A-7EF6-443B-9F61-C7CAEBB32554}">
+  <dimension ref="A1:I52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="53" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" style="53" customWidth="1"/>
+    <col min="12" max="12" width="24.140625" style="47" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MAKLUMAN PELEKAT KENDERAAN PELAJAR BULAN OGOS TAHUN 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+    </row>
+    <row r="2" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="67" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="48"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="112"/>
+      <c r="B3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="112"/>
+      <c r="B4" s="112"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="112"/>
+      <c r="E4" s="112"/>
+      <c r="F4" s="112"/>
+      <c r="G4" s="112"/>
+      <c r="H4" s="112"/>
+      <c r="I4" s="112"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="112"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="112"/>
+      <c r="E5" s="112"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="112"/>
+      <c r="H5" s="112"/>
+      <c r="I5" s="112"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="112"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="112"/>
+      <c r="G6" s="112"/>
+      <c r="H6" s="112"/>
+      <c r="I6" s="112"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="112"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="112"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="112"/>
+      <c r="H7" s="112"/>
+      <c r="I7" s="112"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="112"/>
+      <c r="B8" s="112"/>
+      <c r="C8" s="112"/>
+      <c r="D8" s="112"/>
+      <c r="E8" s="112"/>
+      <c r="F8" s="112"/>
+      <c r="G8" s="112"/>
+      <c r="H8" s="112"/>
+      <c r="I8" s="112"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="112"/>
+      <c r="B9" s="112"/>
+      <c r="C9" s="112"/>
+      <c r="D9" s="112"/>
+      <c r="E9" s="112"/>
+      <c r="F9" s="112"/>
+      <c r="G9" s="112"/>
+      <c r="H9" s="112"/>
+      <c r="I9" s="112"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="112"/>
+      <c r="B10" s="112"/>
+      <c r="C10" s="112"/>
+      <c r="D10" s="112"/>
+      <c r="E10" s="112"/>
+      <c r="F10" s="112"/>
+      <c r="G10" s="112"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="112"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
+      <c r="G11" s="112"/>
+      <c r="H11" s="112"/>
+      <c r="I11" s="112"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="112"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
+      <c r="G12" s="112"/>
+      <c r="H12" s="112"/>
+      <c r="I12" s="112"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="112"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="112"/>
+      <c r="H13" s="112"/>
+      <c r="I13" s="112"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="112"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
+      <c r="G14" s="112"/>
+      <c r="H14" s="112"/>
+      <c r="I14" s="112"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="112"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="112"/>
+      <c r="I15" s="112"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="112"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
+      <c r="G16" s="112"/>
+      <c r="H16" s="112"/>
+      <c r="I16" s="112"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="112"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="112"/>
+      <c r="I17" s="112"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="112"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
+      <c r="G18" s="112"/>
+      <c r="H18" s="112"/>
+      <c r="I18" s="112"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="112"/>
+      <c r="B19" s="112"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
+      <c r="G19" s="112"/>
+      <c r="H19" s="112"/>
+      <c r="I19" s="112"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="112"/>
+      <c r="B20" s="112"/>
+      <c r="C20" s="112"/>
+      <c r="D20" s="112"/>
+      <c r="E20" s="112"/>
+      <c r="F20" s="112"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="112"/>
+      <c r="I20" s="112"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="112"/>
+      <c r="B21" s="112"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="112"/>
+      <c r="E21" s="112"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="112"/>
+      <c r="H21" s="112"/>
+      <c r="I21" s="112"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="112"/>
+      <c r="B22" s="112"/>
+      <c r="C22" s="112"/>
+      <c r="D22" s="112"/>
+      <c r="E22" s="112"/>
+      <c r="F22" s="112"/>
+      <c r="G22" s="112"/>
+      <c r="H22" s="112"/>
+      <c r="I22" s="112"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="112"/>
+      <c r="B23" s="112"/>
+      <c r="C23" s="112"/>
+      <c r="D23" s="112"/>
+      <c r="E23" s="112"/>
+      <c r="F23" s="112"/>
+      <c r="G23" s="112"/>
+      <c r="H23" s="112"/>
+      <c r="I23" s="112"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="112"/>
+      <c r="B24" s="112"/>
+      <c r="C24" s="112"/>
+      <c r="D24" s="112"/>
+      <c r="E24" s="112"/>
+      <c r="F24" s="112"/>
+      <c r="G24" s="112"/>
+      <c r="H24" s="112"/>
+      <c r="I24" s="112"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="112"/>
+      <c r="B25" s="112"/>
+      <c r="C25" s="112"/>
+      <c r="D25" s="112"/>
+      <c r="E25" s="112"/>
+      <c r="F25" s="112"/>
+      <c r="G25" s="112"/>
+      <c r="H25" s="112"/>
+      <c r="I25" s="112"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="112"/>
+      <c r="B26" s="112"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
+      <c r="E26" s="112"/>
+      <c r="F26" s="112"/>
+      <c r="G26" s="112"/>
+      <c r="H26" s="112"/>
+      <c r="I26" s="112"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="112"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
+      <c r="F27" s="112"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="112"/>
+      <c r="I27" s="112"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="112"/>
+      <c r="B28" s="112"/>
+      <c r="C28" s="112"/>
+      <c r="D28" s="112"/>
+      <c r="E28" s="112"/>
+      <c r="F28" s="112"/>
+      <c r="G28" s="112"/>
+      <c r="H28" s="112"/>
+      <c r="I28" s="112"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="112"/>
+      <c r="B29" s="112"/>
+      <c r="C29" s="112"/>
+      <c r="D29" s="112"/>
+      <c r="E29" s="112"/>
+      <c r="F29" s="112"/>
+      <c r="G29" s="112"/>
+      <c r="H29" s="112"/>
+      <c r="I29" s="112"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="112"/>
+      <c r="B30" s="112"/>
+      <c r="C30" s="112"/>
+      <c r="D30" s="112"/>
+      <c r="E30" s="112"/>
+      <c r="F30" s="112"/>
+      <c r="G30" s="112"/>
+      <c r="H30" s="112"/>
+      <c r="I30" s="112"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="112"/>
+      <c r="B31" s="112"/>
+      <c r="C31" s="112"/>
+      <c r="D31" s="112"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="112"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="112"/>
+      <c r="I31" s="112"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="112"/>
+      <c r="B32" s="112"/>
+      <c r="C32" s="112"/>
+      <c r="D32" s="112"/>
+      <c r="E32" s="112"/>
+      <c r="F32" s="112"/>
+      <c r="G32" s="112"/>
+      <c r="H32" s="112"/>
+      <c r="I32" s="112"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="112"/>
+      <c r="B33" s="112"/>
+      <c r="C33" s="112"/>
+      <c r="D33" s="112"/>
+      <c r="E33" s="112"/>
+      <c r="F33" s="112"/>
+      <c r="G33" s="112"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="112"/>
+      <c r="B34" s="112"/>
+      <c r="C34" s="112"/>
+      <c r="D34" s="112"/>
+      <c r="E34" s="112"/>
+      <c r="F34" s="112"/>
+      <c r="G34" s="112"/>
+      <c r="H34" s="112"/>
+      <c r="I34" s="112"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="112"/>
+      <c r="B35" s="112"/>
+      <c r="C35" s="112"/>
+      <c r="D35" s="112"/>
+      <c r="E35" s="112"/>
+      <c r="F35" s="112"/>
+      <c r="G35" s="112"/>
+      <c r="H35" s="112"/>
+      <c r="I35" s="112"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="112"/>
+      <c r="B36" s="112"/>
+      <c r="C36" s="112"/>
+      <c r="D36" s="112"/>
+      <c r="E36" s="112"/>
+      <c r="F36" s="112"/>
+      <c r="G36" s="112"/>
+      <c r="H36" s="112"/>
+      <c r="I36" s="112"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="112"/>
+      <c r="B37" s="112"/>
+      <c r="C37" s="112"/>
+      <c r="D37" s="112"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="112"/>
+      <c r="G37" s="112"/>
+      <c r="H37" s="112"/>
+      <c r="I37" s="112"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="112"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
+      <c r="G38" s="112"/>
+      <c r="H38" s="112"/>
+      <c r="I38" s="112"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="112"/>
+      <c r="B39" s="112"/>
+      <c r="C39" s="112"/>
+      <c r="D39" s="112"/>
+      <c r="E39" s="112"/>
+      <c r="F39" s="112"/>
+      <c r="G39" s="112"/>
+      <c r="H39" s="112"/>
+      <c r="I39" s="112"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="112"/>
+      <c r="B40" s="112"/>
+      <c r="C40" s="112"/>
+      <c r="D40" s="112"/>
+      <c r="E40" s="112"/>
+      <c r="F40" s="112"/>
+      <c r="G40" s="112"/>
+      <c r="H40" s="112"/>
+      <c r="I40" s="112"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="112"/>
+      <c r="B41" s="112"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="112"/>
+      <c r="G41" s="112"/>
+      <c r="H41" s="112"/>
+      <c r="I41" s="112"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="112"/>
+      <c r="B42" s="112"/>
+      <c r="C42" s="112"/>
+      <c r="D42" s="112"/>
+      <c r="E42" s="112"/>
+      <c r="F42" s="112"/>
+      <c r="G42" s="112"/>
+      <c r="H42" s="112"/>
+      <c r="I42" s="112"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="112"/>
+      <c r="B43" s="112"/>
+      <c r="C43" s="112"/>
+      <c r="D43" s="112"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="112"/>
+      <c r="G43" s="112"/>
+      <c r="H43" s="112"/>
+      <c r="I43" s="112"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="112"/>
+      <c r="B44" s="112"/>
+      <c r="C44" s="112"/>
+      <c r="D44" s="112"/>
+      <c r="E44" s="112"/>
+      <c r="F44" s="112"/>
+      <c r="G44" s="112"/>
+      <c r="H44" s="112"/>
+      <c r="I44" s="112"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="112"/>
+      <c r="B45" s="112"/>
+      <c r="C45" s="112"/>
+      <c r="D45" s="112"/>
+      <c r="E45" s="112"/>
+      <c r="F45" s="112"/>
+      <c r="G45" s="112"/>
+      <c r="H45" s="112"/>
+      <c r="I45" s="112"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="112"/>
+      <c r="B46" s="112"/>
+      <c r="C46" s="112"/>
+      <c r="D46" s="112"/>
+      <c r="E46" s="112"/>
+      <c r="F46" s="112"/>
+      <c r="G46" s="112"/>
+      <c r="H46" s="112"/>
+      <c r="I46" s="112"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="112"/>
+      <c r="B47" s="112"/>
+      <c r="C47" s="112"/>
+      <c r="D47" s="112"/>
+      <c r="E47" s="112"/>
+      <c r="F47" s="112"/>
+      <c r="G47" s="112"/>
+      <c r="H47" s="112"/>
+      <c r="I47" s="112"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="112"/>
+      <c r="B48" s="112"/>
+      <c r="C48" s="112"/>
+      <c r="D48" s="112"/>
+      <c r="E48" s="112"/>
+      <c r="F48" s="112"/>
+      <c r="G48" s="112"/>
+      <c r="H48" s="112"/>
+      <c r="I48" s="112"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="112"/>
+      <c r="B49" s="112"/>
+      <c r="C49" s="112"/>
+      <c r="D49" s="112"/>
+      <c r="E49" s="112"/>
+      <c r="F49" s="112"/>
+      <c r="G49" s="112"/>
+      <c r="H49" s="112"/>
+      <c r="I49" s="112"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="112"/>
+      <c r="B50" s="112"/>
+      <c r="C50" s="112"/>
+      <c r="D50" s="112"/>
+      <c r="E50" s="112"/>
+      <c r="F50" s="112"/>
+      <c r="G50" s="112"/>
+      <c r="H50" s="112"/>
+      <c r="I50" s="112"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="112"/>
+      <c r="B51" s="112"/>
+      <c r="C51" s="112"/>
+      <c r="D51" s="112"/>
+      <c r="E51" s="112"/>
+      <c r="F51" s="112"/>
+      <c r="G51" s="112"/>
+      <c r="H51" s="112"/>
+      <c r="I51" s="112"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="112"/>
+      <c r="B52" s="112"/>
+      <c r="C52" s="112"/>
+      <c r="D52" s="112"/>
+      <c r="E52" s="112"/>
+      <c r="F52" s="112"/>
+      <c r="G52" s="112"/>
+      <c r="H52" s="112"/>
+      <c r="I52" s="112"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB8B4E8A-7EF6-443B-9F61-C7CAEBB32554}">
+  <dimension ref="A1:I52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="53" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" style="53" customWidth="1"/>
+    <col min="12" max="12" width="24.140625" style="47" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MAKLUMAN PELEKAT KENDERAAN PELAJAR BULAN SEPTEMBER TAHUN 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+    </row>
+    <row r="2" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="67" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="48"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="112"/>
+      <c r="B3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="112"/>
+      <c r="B4" s="112"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="112"/>
+      <c r="E4" s="112"/>
+      <c r="F4" s="112"/>
+      <c r="G4" s="112"/>
+      <c r="H4" s="112"/>
+      <c r="I4" s="112"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="112"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="112"/>
+      <c r="E5" s="112"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="112"/>
+      <c r="H5" s="112"/>
+      <c r="I5" s="112"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="112"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="112"/>
+      <c r="G6" s="112"/>
+      <c r="H6" s="112"/>
+      <c r="I6" s="112"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="112"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="112"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="112"/>
+      <c r="H7" s="112"/>
+      <c r="I7" s="112"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="112"/>
+      <c r="B8" s="112"/>
+      <c r="C8" s="112"/>
+      <c r="D8" s="112"/>
+      <c r="E8" s="112"/>
+      <c r="F8" s="112"/>
+      <c r="G8" s="112"/>
+      <c r="H8" s="112"/>
+      <c r="I8" s="112"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="112"/>
+      <c r="B9" s="112"/>
+      <c r="C9" s="112"/>
+      <c r="D9" s="112"/>
+      <c r="E9" s="112"/>
+      <c r="F9" s="112"/>
+      <c r="G9" s="112"/>
+      <c r="H9" s="112"/>
+      <c r="I9" s="112"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="112"/>
+      <c r="B10" s="112"/>
+      <c r="C10" s="112"/>
+      <c r="D10" s="112"/>
+      <c r="E10" s="112"/>
+      <c r="F10" s="112"/>
+      <c r="G10" s="112"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="112"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
+      <c r="G11" s="112"/>
+      <c r="H11" s="112"/>
+      <c r="I11" s="112"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="112"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="112"/>
+      <c r="D12" s="112"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="112"/>
+      <c r="G12" s="112"/>
+      <c r="H12" s="112"/>
+      <c r="I12" s="112"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="112"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="112"/>
+      <c r="H13" s="112"/>
+      <c r="I13" s="112"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="112"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="112"/>
+      <c r="D14" s="112"/>
+      <c r="E14" s="112"/>
+      <c r="F14" s="112"/>
+      <c r="G14" s="112"/>
+      <c r="H14" s="112"/>
+      <c r="I14" s="112"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="112"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="112"/>
+      <c r="I15" s="112"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="112"/>
+      <c r="B16" s="112"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
+      <c r="G16" s="112"/>
+      <c r="H16" s="112"/>
+      <c r="I16" s="112"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="112"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="112"/>
+      <c r="I17" s="112"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="112"/>
+      <c r="B18" s="112"/>
+      <c r="C18" s="112"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="112"/>
+      <c r="F18" s="112"/>
+      <c r="G18" s="112"/>
+      <c r="H18" s="112"/>
+      <c r="I18" s="112"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="112"/>
+      <c r="B19" s="112"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
+      <c r="G19" s="112"/>
+      <c r="H19" s="112"/>
+      <c r="I19" s="112"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="112"/>
+      <c r="B20" s="112"/>
+      <c r="C20" s="112"/>
+      <c r="D20" s="112"/>
+      <c r="E20" s="112"/>
+      <c r="F20" s="112"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="112"/>
+      <c r="I20" s="112"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="112"/>
+      <c r="B21" s="112"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="112"/>
+      <c r="E21" s="112"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="112"/>
+      <c r="H21" s="112"/>
+      <c r="I21" s="112"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="112"/>
+      <c r="B22" s="112"/>
+      <c r="C22" s="112"/>
+      <c r="D22" s="112"/>
+      <c r="E22" s="112"/>
+      <c r="F22" s="112"/>
+      <c r="G22" s="112"/>
+      <c r="H22" s="112"/>
+      <c r="I22" s="112"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="112"/>
+      <c r="B23" s="112"/>
+      <c r="C23" s="112"/>
+      <c r="D23" s="112"/>
+      <c r="E23" s="112"/>
+      <c r="F23" s="112"/>
+      <c r="G23" s="112"/>
+      <c r="H23" s="112"/>
+      <c r="I23" s="112"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="112"/>
+      <c r="B24" s="112"/>
+      <c r="C24" s="112"/>
+      <c r="D24" s="112"/>
+      <c r="E24" s="112"/>
+      <c r="F24" s="112"/>
+      <c r="G24" s="112"/>
+      <c r="H24" s="112"/>
+      <c r="I24" s="112"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="112"/>
+      <c r="B25" s="112"/>
+      <c r="C25" s="112"/>
+      <c r="D25" s="112"/>
+      <c r="E25" s="112"/>
+      <c r="F25" s="112"/>
+      <c r="G25" s="112"/>
+      <c r="H25" s="112"/>
+      <c r="I25" s="112"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="112"/>
+      <c r="B26" s="112"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
+      <c r="E26" s="112"/>
+      <c r="F26" s="112"/>
+      <c r="G26" s="112"/>
+      <c r="H26" s="112"/>
+      <c r="I26" s="112"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="112"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
+      <c r="F27" s="112"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="112"/>
+      <c r="I27" s="112"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="112"/>
+      <c r="B28" s="112"/>
+      <c r="C28" s="112"/>
+      <c r="D28" s="112"/>
+      <c r="E28" s="112"/>
+      <c r="F28" s="112"/>
+      <c r="G28" s="112"/>
+      <c r="H28" s="112"/>
+      <c r="I28" s="112"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="112"/>
+      <c r="B29" s="112"/>
+      <c r="C29" s="112"/>
+      <c r="D29" s="112"/>
+      <c r="E29" s="112"/>
+      <c r="F29" s="112"/>
+      <c r="G29" s="112"/>
+      <c r="H29" s="112"/>
+      <c r="I29" s="112"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="112"/>
+      <c r="B30" s="112"/>
+      <c r="C30" s="112"/>
+      <c r="D30" s="112"/>
+      <c r="E30" s="112"/>
+      <c r="F30" s="112"/>
+      <c r="G30" s="112"/>
+      <c r="H30" s="112"/>
+      <c r="I30" s="112"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="112"/>
+      <c r="B31" s="112"/>
+      <c r="C31" s="112"/>
+      <c r="D31" s="112"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="112"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="112"/>
+      <c r="I31" s="112"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="112"/>
+      <c r="B32" s="112"/>
+      <c r="C32" s="112"/>
+      <c r="D32" s="112"/>
+      <c r="E32" s="112"/>
+      <c r="F32" s="112"/>
+      <c r="G32" s="112"/>
+      <c r="H32" s="112"/>
+      <c r="I32" s="112"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="112"/>
+      <c r="B33" s="112"/>
+      <c r="C33" s="112"/>
+      <c r="D33" s="112"/>
+      <c r="E33" s="112"/>
+      <c r="F33" s="112"/>
+      <c r="G33" s="112"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="112"/>
+      <c r="B34" s="112"/>
+      <c r="C34" s="112"/>
+      <c r="D34" s="112"/>
+      <c r="E34" s="112"/>
+      <c r="F34" s="112"/>
+      <c r="G34" s="112"/>
+      <c r="H34" s="112"/>
+      <c r="I34" s="112"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="112"/>
+      <c r="B35" s="112"/>
+      <c r="C35" s="112"/>
+      <c r="D35" s="112"/>
+      <c r="E35" s="112"/>
+      <c r="F35" s="112"/>
+      <c r="G35" s="112"/>
+      <c r="H35" s="112"/>
+      <c r="I35" s="112"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="112"/>
+      <c r="B36" s="112"/>
+      <c r="C36" s="112"/>
+      <c r="D36" s="112"/>
+      <c r="E36" s="112"/>
+      <c r="F36" s="112"/>
+      <c r="G36" s="112"/>
+      <c r="H36" s="112"/>
+      <c r="I36" s="112"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="112"/>
+      <c r="B37" s="112"/>
+      <c r="C37" s="112"/>
+      <c r="D37" s="112"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="112"/>
+      <c r="G37" s="112"/>
+      <c r="H37" s="112"/>
+      <c r="I37" s="112"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="112"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
+      <c r="G38" s="112"/>
+      <c r="H38" s="112"/>
+      <c r="I38" s="112"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="112"/>
+      <c r="B39" s="112"/>
+      <c r="C39" s="112"/>
+      <c r="D39" s="112"/>
+      <c r="E39" s="112"/>
+      <c r="F39" s="112"/>
+      <c r="G39" s="112"/>
+      <c r="H39" s="112"/>
+      <c r="I39" s="112"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="112"/>
+      <c r="B40" s="112"/>
+      <c r="C40" s="112"/>
+      <c r="D40" s="112"/>
+      <c r="E40" s="112"/>
+      <c r="F40" s="112"/>
+      <c r="G40" s="112"/>
+      <c r="H40" s="112"/>
+      <c r="I40" s="112"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="112"/>
+      <c r="B41" s="112"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="112"/>
+      <c r="G41" s="112"/>
+      <c r="H41" s="112"/>
+      <c r="I41" s="112"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="112"/>
+      <c r="B42" s="112"/>
+      <c r="C42" s="112"/>
+      <c r="D42" s="112"/>
+      <c r="E42" s="112"/>
+      <c r="F42" s="112"/>
+      <c r="G42" s="112"/>
+      <c r="H42" s="112"/>
+      <c r="I42" s="112"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="112"/>
+      <c r="B43" s="112"/>
+      <c r="C43" s="112"/>
+      <c r="D43" s="112"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="112"/>
+      <c r="G43" s="112"/>
+      <c r="H43" s="112"/>
+      <c r="I43" s="112"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="112"/>
+      <c r="B44" s="112"/>
+      <c r="C44" s="112"/>
+      <c r="D44" s="112"/>
+      <c r="E44" s="112"/>
+      <c r="F44" s="112"/>
+      <c r="G44" s="112"/>
+      <c r="H44" s="112"/>
+      <c r="I44" s="112"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="112"/>
+      <c r="B45" s="112"/>
+      <c r="C45" s="112"/>
+      <c r="D45" s="112"/>
+      <c r="E45" s="112"/>
+      <c r="F45" s="112"/>
+      <c r="G45" s="112"/>
+      <c r="H45" s="112"/>
+      <c r="I45" s="112"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="112"/>
+      <c r="B46" s="112"/>
+      <c r="C46" s="112"/>
+      <c r="D46" s="112"/>
+      <c r="E46" s="112"/>
+      <c r="F46" s="112"/>
+      <c r="G46" s="112"/>
+      <c r="H46" s="112"/>
+      <c r="I46" s="112"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="112"/>
+      <c r="B47" s="112"/>
+      <c r="C47" s="112"/>
+      <c r="D47" s="112"/>
+      <c r="E47" s="112"/>
+      <c r="F47" s="112"/>
+      <c r="G47" s="112"/>
+      <c r="H47" s="112"/>
+      <c r="I47" s="112"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="112"/>
+      <c r="B48" s="112"/>
+      <c r="C48" s="112"/>
+      <c r="D48" s="112"/>
+      <c r="E48" s="112"/>
+      <c r="F48" s="112"/>
+      <c r="G48" s="112"/>
+      <c r="H48" s="112"/>
+      <c r="I48" s="112"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="112"/>
+      <c r="B49" s="112"/>
+      <c r="C49" s="112"/>
+      <c r="D49" s="112"/>
+      <c r="E49" s="112"/>
+      <c r="F49" s="112"/>
+      <c r="G49" s="112"/>
+      <c r="H49" s="112"/>
+      <c r="I49" s="112"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="112"/>
+      <c r="B50" s="112"/>
+      <c r="C50" s="112"/>
+      <c r="D50" s="112"/>
+      <c r="E50" s="112"/>
+      <c r="F50" s="112"/>
+      <c r="G50" s="112"/>
+      <c r="H50" s="112"/>
+      <c r="I50" s="112"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="112"/>
+      <c r="B51" s="112"/>
+      <c r="C51" s="112"/>
+      <c r="D51" s="112"/>
+      <c r="E51" s="112"/>
+      <c r="F51" s="112"/>
+      <c r="G51" s="112"/>
+      <c r="H51" s="112"/>
+      <c r="I51" s="112"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="112"/>
+      <c r="B52" s="112"/>
+      <c r="C52" s="112"/>
+      <c r="D52" s="112"/>
+      <c r="E52" s="112"/>
+      <c r="F52" s="112"/>
+      <c r="G52" s="112"/>
+      <c r="H52" s="112"/>
+      <c r="I52" s="112"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61372893-D864-4FC7-857F-581210142782}">
   <dimension ref="A1:I52"/>

</xml_diff>